<commit_message>
Fix KHL playoff Excel template structure
</commit_message>
<xml_diff>
--- a/templates/khl-playoff-data-template.xlsx
+++ b/templates/khl-playoff-data-template.xlsx
@@ -1,5 +1,5 @@
 
-<file path=xl\workbook.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <sheets>
     <sheet name="KHL playoff data" sheetId="1" r:id="rId1"/>
@@ -8,7 +8,32 @@
 </workbook>
 </file>
 
-<file path=xl\worksheets\sheet1.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <fonts count="1">
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+    </font>
+  </fonts>
+  <fills count="1">
+    <fill>
+      <patternFill patternType="none"/>
+    </fill>
+  </fills>
+  <borders count="1">
+    <border/>
+  </borders>
+  <cellStyleXfs count="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
+  </cellStyleXfs>
+  <cellXfs count="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+  </cellXfs>
+</styleSheet>
+</file>
+
+<file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetData>
     <row r="1">
@@ -149,7 +174,7 @@
 </worksheet>
 </file>
 
-<file path=xl\worksheets\sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetData>
     <row r="1">

</xml_diff>